<commit_message>
prg Mon Jun  1 06:31:03 PM CEST 2026
</commit_message>
<xml_diff>
--- a/public/routers/A0_Sistema_FV/A61_Conectado_a_red/FV03_pvgis6.xlsx
+++ b/public/routers/A0_Sistema_FV/A61_Conectado_a_red/FV03_pvgis6.xlsx
@@ -967,7 +967,7 @@
       </c>
       <c r="AF2" t="inlineStr">
         <is>
-          <t>[1,1,1,1,1,1,1,1,1,1,1,1,1,1,1,1]</t>
+          <t>[1,1,40,45,50,55,1,1,1,1,1,1,1,1,1,1]</t>
         </is>
       </c>
       <c r="AG2" t="inlineStr">
@@ -1499,7 +1499,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G12"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1525,15 +1525,10 @@
       </c>
       <c r="E1" s="1" t="inlineStr">
         <is>
-          <t>valor</t>
+          <t>€/Wdc</t>
         </is>
       </c>
       <c r="F1" s="1" t="inlineStr">
-        <is>
-          <t>Variable_Ud</t>
-        </is>
-      </c>
-      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>MO (%)</t>
         </is>
@@ -1561,12 +1556,7 @@
       <c r="E2" t="n">
         <v>0.22</v>
       </c>
-      <c r="F2" t="inlineStr">
-        <is>
-          <t>€/Wdc</t>
-        </is>
-      </c>
-      <c r="G2" t="n">
+      <c r="F2" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1592,12 +1582,7 @@
       <c r="E3" t="n">
         <v>0.12</v>
       </c>
-      <c r="F3" t="inlineStr">
-        <is>
-          <t>€/Wdc</t>
-        </is>
-      </c>
-      <c r="G3" t="n">
+      <c r="F3" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1623,12 +1608,7 @@
       <c r="E4" t="n">
         <v>0.15</v>
       </c>
-      <c r="F4" t="inlineStr">
-        <is>
-          <t>€/kWh</t>
-        </is>
-      </c>
-      <c r="G4" t="n">
+      <c r="F4" t="n">
         <v>5</v>
       </c>
     </row>
@@ -1654,12 +1634,7 @@
       <c r="E5" t="n">
         <v>0.19</v>
       </c>
-      <c r="F5" t="inlineStr">
-        <is>
-          <t>€/Wdc</t>
-        </is>
-      </c>
-      <c r="G5" t="n">
+      <c r="F5" t="n">
         <v>40</v>
       </c>
     </row>
@@ -1685,12 +1660,7 @@
       <c r="E6" t="n">
         <v>0.02</v>
       </c>
-      <c r="F6" t="inlineStr">
-        <is>
-          <t>€/Wdc</t>
-        </is>
-      </c>
-      <c r="G6" t="n">
+      <c r="F6" t="n">
         <v>10</v>
       </c>
     </row>
@@ -1716,12 +1686,7 @@
       <c r="E7" t="n">
         <v>0.005</v>
       </c>
-      <c r="F7" t="inlineStr">
-        <is>
-          <t>€/Wdc</t>
-        </is>
-      </c>
-      <c r="G7" t="n">
+      <c r="F7" t="n">
         <v>80</v>
       </c>
     </row>
@@ -1747,12 +1712,7 @@
       <c r="E8" t="n">
         <v>0.02</v>
       </c>
-      <c r="F8" t="inlineStr">
-        <is>
-          <t>€/Wdc</t>
-        </is>
-      </c>
-      <c r="G8" t="n">
+      <c r="F8" t="n">
         <v>100</v>
       </c>
     </row>
@@ -1778,12 +1738,7 @@
       <c r="E9" t="n">
         <v>0.01</v>
       </c>
-      <c r="F9" t="inlineStr">
-        <is>
-          <t>€/Wdc</t>
-        </is>
-      </c>
-      <c r="G9" t="n">
+      <c r="F9" t="n">
         <v>90</v>
       </c>
     </row>
@@ -1809,12 +1764,7 @@
       <c r="E10" t="n">
         <v>0.18</v>
       </c>
-      <c r="F10" t="inlineStr">
-        <is>
-          <t>€/Wdc</t>
-        </is>
-      </c>
-      <c r="G10" t="n">
+      <c r="F10" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1840,12 +1790,7 @@
       <c r="E11" t="n">
         <v>0.04</v>
       </c>
-      <c r="F11" t="inlineStr">
-        <is>
-          <t>€/Wdc</t>
-        </is>
-      </c>
-      <c r="G11" t="n">
+      <c r="F11" t="n">
         <v>0</v>
       </c>
     </row>
@@ -1871,12 +1816,7 @@
       <c r="E12" t="n">
         <v>0</v>
       </c>
-      <c r="F12" t="inlineStr">
-        <is>
-          <t>@</t>
-        </is>
-      </c>
-      <c r="G12" t="n">
+      <c r="F12" t="n">
         <v>0</v>
       </c>
     </row>

</xml_diff>